<commit_message>
feat: data analysis developed; draft report prepared
</commit_message>
<xml_diff>
--- a/src/ANALYSIS/normalized_numerical_data.xlsx
+++ b/src/ANALYSIS/normalized_numerical_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HARDPC\Desktop\github\riotdev\src\ANALYSIS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86E5D04E-D351-4EC4-8E33-A8C96071DC17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C72B872A-0FCD-4783-94EF-45A7302B33E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -908,8 +908,19 @@
   <dimension ref="A1:BD201"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="22" max="22" width="12" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="23.5703125" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="12" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="20" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="27.140625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="29.85546875" bestFit="1" customWidth="1"/>
     <col min="39" max="39" width="17.85546875" bestFit="1" customWidth="1"/>
     <col min="40" max="40" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="24.7109375" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="16.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:56" x14ac:dyDescent="0.25">

</xml_diff>